<commit_message>
traubajos con la orden de materia prima especificamente cerrar documentos
</commit_message>
<xml_diff>
--- a/bin/Debug/net8.0-windows10.0.19041/Template.xlsx
+++ b/bin/Debug/net8.0-windows10.0.19041/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29024"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programacion\Ritrama2025\bin\Debug\net8.0-windows10.0.19041\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A01C3C6E-7ED1-4DBD-8285-47A601039684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606170CE-A23C-47CB-9150-8C9D46C8E519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32580" yWindow="3945" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32940" yWindow="2490" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TemplateMateriaPrima" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="22">
   <si>
     <t>Product. Id.</t>
   </si>
@@ -86,15 +86,6 @@
   </si>
   <si>
     <t>05070</t>
-  </si>
-  <si>
-    <t>06235</t>
-  </si>
-  <si>
-    <t>06274</t>
-  </si>
-  <si>
-    <t>06701</t>
   </si>
 </sst>
 </file>
@@ -434,18 +425,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" customWidth="1"/>
+    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.140625" customWidth="1"/>
+    <col min="7" max="7" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -789,84 +780,6 @@
         <v>12504163</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14">
-        <v>17</v>
-      </c>
-      <c r="E14">
-        <v>19800</v>
-      </c>
-      <c r="F14">
-        <v>300</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>121000141</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15">
-        <v>18</v>
-      </c>
-      <c r="E15">
-        <v>20000</v>
-      </c>
-      <c r="F15">
-        <v>350</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>12504471</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16">
-        <v>20</v>
-      </c>
-      <c r="E16">
-        <v>40000</v>
-      </c>
-      <c r="F16">
-        <v>378</v>
-      </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>12556001</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>

</xml_diff>